<commit_message>
docs(hw03): prepare evidence-gated usability sessions
</commit_message>
<xml_diff>
--- a/docs/assignments/HW03/deliverables/usability/sus_survey_results.xlsx
+++ b/docs/assignments/HW03/deliverables/usability/sus_survey_results.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'SUS Results'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'SUS Results'!$A$1:$R$9</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -563,16 +563,21 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="L2" s="2">
+        <f>IF(COUNTA(B2:K2)=0,"",IF(COUNTA(B2:K2)&lt;10,"INCOMPLETE",SUM(B2-1,5-C2,D2-1,5-E2,F2-1,5-G2,H2-1,5-I2,J2-1,5-K2)))</f>
+        <v/>
+      </c>
+      <c r="M2" s="2">
+        <f>IF(ISNUMBER(L2),L2*2.5,"")</f>
+        <v/>
+      </c>
       <c r="N2" s="2" t="inlineStr"/>
       <c r="O2" s="2" t="inlineStr"/>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>Not collected</t>
-        </is>
+      <c r="R2" s="2">
+        <f>IF(COUNTA(B2:K2)=0,"Not collected",IF(COUNTA(B2:K2)&lt;10,"Incomplete","Calculated"))</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -591,16 +596,21 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="L3" s="2">
+        <f>IF(COUNTA(B3:K3)=0,"",IF(COUNTA(B3:K3)&lt;10,"INCOMPLETE",SUM(B3-1,5-C3,D3-1,5-E3,F3-1,5-G3,H3-1,5-I3,J3-1,5-K3)))</f>
+        <v/>
+      </c>
+      <c r="M3" s="2">
+        <f>IF(ISNUMBER(L3),L3*2.5,"")</f>
+        <v/>
+      </c>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Not collected</t>
-        </is>
+      <c r="R3" s="2">
+        <f>IF(COUNTA(B3:K3)=0,"Not collected",IF(COUNTA(B3:K3)&lt;10,"Incomplete","Calculated"))</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -619,16 +629,21 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="L4" s="2">
+        <f>IF(COUNTA(B4:K4)=0,"",IF(COUNTA(B4:K4)&lt;10,"INCOMPLETE",SUM(B4-1,5-C4,D4-1,5-E4,F4-1,5-G4,H4-1,5-I4,J4-1,5-K4)))</f>
+        <v/>
+      </c>
+      <c r="M4" s="2">
+        <f>IF(ISNUMBER(L4),L4*2.5,"")</f>
+        <v/>
+      </c>
       <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
       <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>Not collected</t>
-        </is>
+      <c r="R4" s="2">
+        <f>IF(COUNTA(B4:K4)=0,"Not collected",IF(COUNTA(B4:K4)&lt;10,"Incomplete","Calculated"))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -647,16 +662,21 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
+      <c r="L5" s="2">
+        <f>IF(COUNTA(B5:K5)=0,"",IF(COUNTA(B5:K5)&lt;10,"INCOMPLETE",SUM(B5-1,5-C5,D5-1,5-E5,F5-1,5-G5,H5-1,5-I5,J5-1,5-K5)))</f>
+        <v/>
+      </c>
+      <c r="M5" s="2">
+        <f>IF(ISNUMBER(L5),L5*2.5,"")</f>
+        <v/>
+      </c>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
       <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>Not collected</t>
-        </is>
+      <c r="R5" s="2">
+        <f>IF(COUNTA(B5:K5)=0,"Not collected",IF(COUNTA(B5:K5)&lt;10,"Incomplete","Calculated"))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -675,16 +695,21 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="L6" s="2">
+        <f>IF(COUNTA(B6:K6)=0,"",IF(COUNTA(B6:K6)&lt;10,"INCOMPLETE",SUM(B6-1,5-C6,D6-1,5-E6,F6-1,5-G6,H6-1,5-I6,J6-1,5-K6)))</f>
+        <v/>
+      </c>
+      <c r="M6" s="2">
+        <f>IF(ISNUMBER(L6),L6*2.5,"")</f>
+        <v/>
+      </c>
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
       <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>Not collected</t>
-        </is>
+      <c r="R6" s="2">
+        <f>IF(COUNTA(B6:K6)=0,"Not collected",IF(COUNTA(B6:K6)&lt;10,"Incomplete","Calculated"))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -703,16 +728,21 @@
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+      <c r="L7" s="2">
+        <f>IF(COUNTA(B7:K7)=0,"",IF(COUNTA(B7:K7)&lt;10,"INCOMPLETE",SUM(B7-1,5-C7,D7-1,5-E7,F7-1,5-G7,H7-1,5-I7,J7-1,5-K7)))</f>
+        <v/>
+      </c>
+      <c r="M7" s="2">
+        <f>IF(ISNUMBER(L7),L7*2.5,"")</f>
+        <v/>
+      </c>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
       <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>Not collected</t>
-        </is>
+      <c r="R7" s="2">
+        <f>IF(COUNTA(B7:K7)=0,"Not collected",IF(COUNTA(B7:K7)&lt;10,"Incomplete","Calculated"))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -731,16 +761,21 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="L8" s="2">
+        <f>IF(COUNTA(B8:K8)=0,"",IF(COUNTA(B8:K8)&lt;10,"INCOMPLETE",SUM(B8-1,5-C8,D8-1,5-E8,F8-1,5-G8,H8-1,5-I8,J8-1,5-K8)))</f>
+        <v/>
+      </c>
+      <c r="M8" s="2">
+        <f>IF(ISNUMBER(L8),L8*2.5,"")</f>
+        <v/>
+      </c>
       <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
       <c r="Q8" s="2" t="inlineStr"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Not collected</t>
-        </is>
+      <c r="R8" s="2">
+        <f>IF(COUNTA(B8:K8)=0,"Not collected",IF(COUNTA(B8:K8)&lt;10,"Incomplete","Calculated"))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -760,19 +795,27 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="2" t="inlineStr"/>
+      <c r="M9" s="2">
+        <f>IF(COUNT(M2:M8)=7,AVERAGE(M2:M8),"")</f>
+        <v/>
+      </c>
       <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
       <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>Not calculated</t>
-        </is>
+      <c r="R9" s="2">
+        <f>IF(COUNT(M2:M8)=7,"Calculated","Not calculated")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:R9"/>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:K8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid SUS response" error="Enter a whole-number SUS response from 1 to 5." promptTitle="SUS response" prompt="Enter 1 (strongly disagree) through 5 (strongly agree)." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>